<commit_message>
notes/costs: the Mistral note in the kind column
</commit_message>
<xml_diff>
--- a/notes/costs/vision_models_2026-09-28.xlsx
+++ b/notes/costs/vision_models_2026-09-28.xlsx
@@ -11250,11 +11250,7 @@
           <t>Mistral: Mistral Medium 3.5</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>cache read 10% per Mistral (not on OpenRouter)</t>
-        </is>
-      </c>
+      <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
           <t>yes</t>
@@ -11267,6 +11263,11 @@
       </c>
       <c r="F180" s="10" t="n">
         <v>262144</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>cache read 10% per Mistral (not on OpenRouter)</t>
+        </is>
       </c>
       <c r="H180" s="11" t="n">
         <v>1.5</v>

</xml_diff>